<commit_message>
Add investment cost from PyPSA to VRES & ThermalGen, update DataSource
Switch to newest InOutModule
</commit_message>
<xml_diff>
--- a/data/NREL-118/Power_VRES.xlsx
+++ b/data/NREL-118/Power_VRES.xlsx
@@ -1172,19 +1172,19 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="14" t="n">
         <v>746.76</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K8" s="15" t="n">
         <v>0.01</v>
@@ -1245,19 +1245,19 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>369.26</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K9" s="15" t="n">
         <v>0.01</v>
@@ -1318,19 +1318,19 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="14" t="n">
         <v>264.47</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K10" s="15" t="n">
         <v>0.01</v>
@@ -1391,19 +1391,19 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>4.85</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K11" s="15" t="n">
         <v>0.01</v>
@@ -1464,19 +1464,19 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>0.12</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K12" s="15" t="n">
         <v>0.01</v>
@@ -1537,19 +1537,19 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>6.33</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K13" s="15" t="n">
         <v>0.01</v>
@@ -1610,19 +1610,19 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>0.21</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K14" s="15" t="n">
         <v>0.01</v>
@@ -1683,19 +1683,19 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>2.51</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K15" s="15" t="n">
         <v>0.01</v>
@@ -1756,19 +1756,19 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>12.85</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K16" s="15" t="n">
         <v>0.01</v>
@@ -1829,19 +1829,19 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>9.710000000000001</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K17" s="15" t="n">
         <v>0.01</v>
@@ -1902,19 +1902,19 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>1.98</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K18" s="15" t="n">
         <v>0.01</v>
@@ -1975,19 +1975,19 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="14" t="n">
         <v>1.54</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K19" s="15" t="n">
         <v>0.01</v>
@@ -2048,19 +2048,19 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="14" t="n">
         <v>0.26</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K20" s="15" t="n">
         <v>0.01</v>
@@ -2121,19 +2121,19 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="14" t="n">
         <v>11.71</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K21" s="15" t="n">
         <v>0.01</v>
@@ -2194,19 +2194,19 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="14" t="n">
         <v>10.53</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K22" s="15" t="n">
         <v>0.01</v>
@@ -2267,19 +2267,19 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="14" t="n">
         <v>6.6</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K23" s="15" t="n">
         <v>0.01</v>
@@ -2340,19 +2340,19 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>3.01</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K24" s="15" t="n">
         <v>0.01</v>
@@ -2413,19 +2413,19 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" s="14" t="n">
         <v>12.35</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K25" s="15" t="n">
         <v>0.01</v>
@@ -2486,19 +2486,19 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" s="14" t="n">
         <v>0.1</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K26" s="15" t="n">
         <v>0.01</v>
@@ -2559,19 +2559,19 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>10.08</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K27" s="15" t="n">
         <v>0.01</v>
@@ -2632,19 +2632,19 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>18.42</v>
       </c>
       <c r="H28" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K28" s="15" t="n">
         <v>0.01</v>
@@ -2705,19 +2705,19 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>8.98</v>
       </c>
       <c r="H29" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K29" s="15" t="n">
         <v>0.01</v>
@@ -2778,19 +2778,19 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>0.29</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K30" s="15" t="n">
         <v>0.01</v>
@@ -2851,19 +2851,19 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" s="14" t="n">
         <v>1.45</v>
       </c>
       <c r="H31" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K31" s="15" t="n">
         <v>0.01</v>
@@ -2924,19 +2924,19 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="14" t="n">
         <v>1.94</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K32" s="15" t="n">
         <v>0.01</v>
@@ -2997,19 +2997,19 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" s="14" t="n">
         <v>1.8</v>
       </c>
       <c r="H33" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K33" s="15" t="n">
         <v>0.01</v>
@@ -3070,19 +3070,19 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" s="14" t="n">
         <v>1.13</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K34" s="15" t="n">
         <v>0.01</v>
@@ -3143,19 +3143,19 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" s="14" t="n">
         <v>8.029999999999999</v>
       </c>
       <c r="H35" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K35" s="15" t="n">
         <v>0.01</v>
@@ -3216,19 +3216,19 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>8.630000000000001</v>
       </c>
       <c r="H36" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K36" s="15" t="n">
         <v>0.01</v>
@@ -3289,19 +3289,19 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="14" t="n">
         <v>4.5</v>
       </c>
       <c r="H37" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K37" s="15" t="n">
         <v>0.01</v>
@@ -3362,19 +3362,19 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="14" t="n">
         <v>116.03</v>
       </c>
       <c r="H38" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K38" s="15" t="n">
         <v>0.01</v>
@@ -3435,19 +3435,19 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" s="14" t="n">
         <v>173.97</v>
       </c>
       <c r="H39" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K39" s="15" t="n">
         <v>0.01</v>
@@ -3508,19 +3508,19 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>132</v>
       </c>
       <c r="H40" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K40" s="15" t="n">
         <v>0.01</v>
@@ -3581,19 +3581,19 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" s="14" t="n">
         <v>125</v>
       </c>
       <c r="H41" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I41" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K41" s="15" t="n">
         <v>0.01</v>
@@ -3654,19 +3654,19 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>45</v>
       </c>
       <c r="H42" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K42" s="15" t="n">
         <v>0.01</v>
@@ -3727,19 +3727,19 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="14" t="n">
         <v>128.9</v>
       </c>
       <c r="H43" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K43" s="15" t="n">
         <v>0.01</v>
@@ -3800,19 +3800,19 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" s="14" t="n">
         <v>26</v>
       </c>
       <c r="H44" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K44" s="15" t="n">
         <v>0.01</v>
@@ -3873,19 +3873,19 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="14" t="n">
         <v>20</v>
       </c>
       <c r="H45" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I45" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K45" s="15" t="n">
         <v>0.01</v>
@@ -3946,19 +3946,19 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H46" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I46" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K46" s="15" t="n">
         <v>0.01</v>
@@ -4019,19 +4019,19 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H47" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J47" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K47" s="15" t="n">
         <v>0.01</v>
@@ -4092,19 +4092,19 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G48" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H48" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K48" s="15" t="n">
         <v>0.01</v>
@@ -4165,19 +4165,19 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H49" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K49" s="15" t="n">
         <v>0.01</v>
@@ -4238,19 +4238,19 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H50" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K50" s="15" t="n">
         <v>0.01</v>
@@ -4311,19 +4311,19 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H51" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K51" s="15" t="n">
         <v>0.01</v>
@@ -4384,19 +4384,19 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H52" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K52" s="15" t="n">
         <v>0.01</v>
@@ -4457,19 +4457,19 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H53" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J53" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K53" s="15" t="n">
         <v>0.01</v>
@@ -4530,19 +4530,19 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G54" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H54" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K54" s="15" t="n">
         <v>0.01</v>
@@ -4603,19 +4603,19 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55" s="14" t="n">
         <v>1.75</v>
       </c>
       <c r="H55" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K55" s="15" t="n">
         <v>0.01</v>
@@ -4676,19 +4676,19 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G56" s="14" t="n">
         <v>1.1</v>
       </c>
       <c r="H56" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I56" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K56" s="15" t="n">
         <v>0.01</v>
@@ -4749,19 +4749,19 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="14" t="n">
         <v>4.69</v>
       </c>
       <c r="H57" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I57" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J57" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K57" s="15" t="n">
         <v>0.01</v>
@@ -4822,19 +4822,19 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="14" t="n">
         <v>15.65</v>
       </c>
       <c r="H58" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K58" s="15" t="n">
         <v>0.01</v>
@@ -4895,19 +4895,19 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>10.64</v>
       </c>
       <c r="H59" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I59" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K59" s="15" t="n">
         <v>0.01</v>
@@ -4968,19 +4968,19 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>16.09</v>
       </c>
       <c r="H60" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I60" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K60" s="15" t="n">
         <v>0.01</v>
@@ -5041,19 +5041,19 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" s="14" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="H61" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I61" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K61" s="15" t="n">
         <v>0.01</v>
@@ -5114,19 +5114,19 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G62" s="14" t="n">
         <v>20.01</v>
       </c>
       <c r="H62" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K62" s="15" t="n">
         <v>0.01</v>
@@ -5187,19 +5187,19 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" s="14" t="n">
         <v>20.07</v>
       </c>
       <c r="H63" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I63" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K63" s="15" t="n">
         <v>0.01</v>
@@ -5260,19 +5260,19 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" s="14" t="n">
         <v>6.84</v>
       </c>
       <c r="H64" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K64" s="15" t="n">
         <v>0.01</v>
@@ -5333,19 +5333,19 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" s="14" t="n">
         <v>8.01</v>
       </c>
       <c r="H65" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J65" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K65" s="15" t="n">
         <v>0.01</v>
@@ -5406,19 +5406,19 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" s="14" t="n">
         <v>12.42</v>
       </c>
       <c r="H66" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J66" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K66" s="15" t="n">
         <v>0.01</v>
@@ -5479,19 +5479,19 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G67" s="14" t="n">
         <v>15.89</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K67" s="15" t="n">
         <v>0.01</v>
@@ -5552,19 +5552,19 @@
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G68" s="14" t="n">
         <v>1.97</v>
       </c>
       <c r="H68" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I68" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J68" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K68" s="15" t="n">
         <v>0.01</v>
@@ -5625,19 +5625,19 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" s="14" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="H69" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I69" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K69" s="15" t="n">
         <v>0.01</v>
@@ -5698,19 +5698,19 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G70" s="14" t="n">
         <v>60</v>
       </c>
       <c r="H70" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I70" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K70" s="15" t="n">
         <v>0.01</v>
@@ -5771,19 +5771,19 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G71" s="14" t="n">
         <v>21</v>
       </c>
       <c r="H71" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I71" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K71" s="15" t="n">
         <v>0.01</v>
@@ -5844,19 +5844,19 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G72" s="14" t="n">
         <v>64.8</v>
       </c>
       <c r="H72" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I72" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K72" s="15" t="n">
         <v>0.01</v>
@@ -5917,19 +5917,19 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G73" s="14" t="n">
         <v>123.5</v>
       </c>
       <c r="H73" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J73" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K73" s="15" t="n">
         <v>0.01</v>
@@ -5990,19 +5990,19 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" s="14" t="n">
         <v>40</v>
       </c>
       <c r="H74" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I74" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K74" s="15" t="n">
         <v>0.01</v>
@@ -6063,19 +6063,19 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G75" s="14" t="n">
         <v>96</v>
       </c>
       <c r="H75" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I75" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J75" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K75" s="15" t="n">
         <v>0.01</v>
@@ -6136,19 +6136,19 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G76" s="14" t="n">
         <v>123</v>
       </c>
       <c r="H76" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I76" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K76" s="15" t="n">
         <v>0.01</v>
@@ -6209,19 +6209,19 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G77" s="14" t="n">
         <v>150</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I77" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J77" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K77" s="15" t="n">
         <v>0.01</v>
@@ -6282,19 +6282,19 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78" s="14" t="n">
         <v>104.99</v>
       </c>
       <c r="H78" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I78" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K78" s="15" t="n">
         <v>0.01</v>
@@ -6355,19 +6355,19 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G79" s="14" t="n">
         <v>25.2</v>
       </c>
       <c r="H79" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I79" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J79" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K79" s="15" t="n">
         <v>0.01</v>
@@ -6428,19 +6428,19 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G80" s="14" t="n">
         <v>25</v>
       </c>
       <c r="H80" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I80" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J80" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K80" s="15" t="n">
         <v>0.01</v>
@@ -6501,19 +6501,19 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G81" s="14" t="n">
         <v>25</v>
       </c>
       <c r="H81" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I81" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J81" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K81" s="15" t="n">
         <v>0.01</v>
@@ -6574,19 +6574,19 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G82" s="14" t="n">
         <v>30</v>
       </c>
       <c r="H82" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I82" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J82" s="15" t="n">
-        <v>0</v>
+        <v>38283.38018933929</v>
       </c>
       <c r="K82" s="15" t="n">
         <v>0.01</v>
@@ -6647,19 +6647,19 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G83" s="14" t="n">
         <v>11.5</v>
       </c>
       <c r="H83" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I83" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K83" s="15" t="n">
         <v>0.05</v>
@@ -6720,19 +6720,19 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84" s="14" t="n">
         <v>38</v>
       </c>
       <c r="H84" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J84" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K84" s="15" t="n">
         <v>0.05</v>
@@ -6793,19 +6793,19 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85" s="14" t="n">
         <v>10</v>
       </c>
       <c r="H85" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I85" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J85" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K85" s="15" t="n">
         <v>0.05</v>
@@ -6866,19 +6866,19 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G86" s="14" t="n">
         <v>5</v>
       </c>
       <c r="H86" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I86" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J86" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K86" s="15" t="n">
         <v>0.05</v>
@@ -6939,19 +6939,19 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G87" s="14" t="n">
         <v>1.1</v>
       </c>
       <c r="H87" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I87" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J87" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K87" s="15" t="n">
         <v>0.05</v>
@@ -7012,19 +7012,19 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88" s="14" t="n">
         <v>24.1</v>
       </c>
       <c r="H88" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I88" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J88" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K88" s="15" t="n">
         <v>0.05</v>
@@ -7085,19 +7085,19 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G89" s="14" t="n">
         <v>16.6</v>
       </c>
       <c r="H89" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I89" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J89" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K89" s="15" t="n">
         <v>0.05</v>
@@ -7158,19 +7158,19 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90" s="14" t="n">
         <v>16.6</v>
       </c>
       <c r="H90" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I90" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J90" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K90" s="15" t="n">
         <v>0.05</v>
@@ -7231,19 +7231,19 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91" s="14" t="n">
         <v>16.6</v>
       </c>
       <c r="H91" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I91" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K91" s="15" t="n">
         <v>0.05</v>
@@ -7304,19 +7304,19 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G92" s="14" t="n">
         <v>16.6</v>
       </c>
       <c r="H92" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I92" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K92" s="15" t="n">
         <v>0.05</v>
@@ -7377,19 +7377,19 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" s="14" t="n">
         <v>16.6</v>
       </c>
       <c r="H93" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J93" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K93" s="15" t="n">
         <v>0.05</v>
@@ -7450,19 +7450,19 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G94" s="14" t="n">
         <v>97.5</v>
       </c>
       <c r="H94" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I94" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K94" s="15" t="n">
         <v>0.05</v>
@@ -7523,19 +7523,19 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G95" s="14" t="n">
         <v>58.7</v>
       </c>
       <c r="H95" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I95" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J95" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K95" s="15" t="n">
         <v>0.05</v>
@@ -7596,19 +7596,19 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G96" s="14" t="n">
         <v>400</v>
       </c>
       <c r="H96" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I96" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J96" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K96" s="15" t="n">
         <v>0.05</v>
@@ -7669,19 +7669,19 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97" s="14" t="n">
         <v>50</v>
       </c>
       <c r="H97" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I97" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J97" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K97" s="15" t="n">
         <v>0.05</v>
@@ -7742,19 +7742,19 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G98" s="14" t="n">
         <v>149.5</v>
       </c>
       <c r="H98" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I98" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J98" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K98" s="15" t="n">
         <v>0.05</v>
@@ -7815,19 +7815,19 @@
         </is>
       </c>
       <c r="F99" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G99" s="14" t="n">
         <v>149.5</v>
       </c>
       <c r="H99" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I99" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J99" s="15" t="n">
-        <v>0</v>
+        <v>101644.123323877</v>
       </c>
       <c r="K99" s="15" t="n">
         <v>0.05</v>

</xml_diff>

<commit_message>
Set RoR-Plants to be investment candidates
</commit_message>
<xml_diff>
--- a/data/NREL-118/Power_VRES.xlsx
+++ b/data/NREL-118/Power_VRES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo\data\NREL-118\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849F1623-ABA0-43A6-A7ED-359ED923BCBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E7F234-070B-4EE4-B0F7-FC09BD881AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34230" yWindow="-21705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4170" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenarioA" sheetId="1" r:id="rId1"/>
@@ -6146,16 +6146,16 @@
         <v>74</v>
       </c>
       <c r="F100" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G100" s="14">
         <v>0.8</v>
       </c>
       <c r="H100" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I100" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J100" s="15">
         <f>2336*1000/100</f>
@@ -6194,16 +6194,16 @@
         <v>119</v>
       </c>
       <c r="F101" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G101" s="14">
         <v>1.35</v>
       </c>
       <c r="H101" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I101" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J101" s="15">
         <f t="shared" ref="J101:J127" si="4">2336*1000/100</f>
@@ -6242,16 +6242,16 @@
         <v>119</v>
       </c>
       <c r="F102" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G102" s="14">
         <v>4.6500000000000004</v>
       </c>
       <c r="H102" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I102" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J102" s="15">
         <f t="shared" si="4"/>
@@ -6290,16 +6290,16 @@
         <v>191</v>
       </c>
       <c r="F103" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G103" s="14">
         <v>648.44000000000005</v>
       </c>
       <c r="H103" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I103" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J103" s="15">
         <f t="shared" si="4"/>
@@ -6338,16 +6338,16 @@
         <v>193</v>
       </c>
       <c r="F104" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G104" s="14">
         <v>765.77</v>
       </c>
       <c r="H104" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I104" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J104" s="15">
         <f t="shared" si="4"/>
@@ -6386,16 +6386,16 @@
         <v>195</v>
       </c>
       <c r="F105" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" s="14">
         <v>765.77</v>
       </c>
       <c r="H105" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I105" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J105" s="15">
         <f t="shared" si="4"/>
@@ -6434,16 +6434,16 @@
         <v>195</v>
       </c>
       <c r="F106" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G106" s="14">
         <v>765.77</v>
       </c>
       <c r="H106" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I106" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J106" s="15">
         <f t="shared" si="4"/>
@@ -6482,16 +6482,16 @@
         <v>146</v>
       </c>
       <c r="F107" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G107" s="14">
         <v>742.63</v>
       </c>
       <c r="H107" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I107" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J107" s="15">
         <f t="shared" si="4"/>
@@ -6530,16 +6530,16 @@
         <v>146</v>
       </c>
       <c r="F108" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G108" s="14">
         <v>742.63</v>
       </c>
       <c r="H108" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I108" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J108" s="15">
         <f t="shared" si="4"/>
@@ -6578,16 +6578,16 @@
         <v>200</v>
       </c>
       <c r="F109" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G109" s="14">
         <v>286.45999999999998</v>
       </c>
       <c r="H109" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I109" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J109" s="15">
         <f t="shared" si="4"/>
@@ -6626,16 +6626,16 @@
         <v>191</v>
       </c>
       <c r="F110" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110" s="14">
         <v>286.45999999999998</v>
       </c>
       <c r="H110" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110" s="15">
         <f t="shared" si="4"/>
@@ -6674,16 +6674,16 @@
         <v>203</v>
       </c>
       <c r="F111" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111" s="14">
         <v>286.45999999999998</v>
       </c>
       <c r="H111" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I111" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111" s="15">
         <f t="shared" si="4"/>
@@ -6722,16 +6722,16 @@
         <v>203</v>
       </c>
       <c r="F112" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G112" s="14">
         <v>1116.06</v>
       </c>
       <c r="H112" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I112" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J112" s="15">
         <f t="shared" si="4"/>
@@ -6770,16 +6770,16 @@
         <v>203</v>
       </c>
       <c r="F113" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G113" s="14">
         <v>1116.06</v>
       </c>
       <c r="H113" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I113" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J113" s="15">
         <f t="shared" si="4"/>
@@ -6818,16 +6818,16 @@
         <v>207</v>
       </c>
       <c r="F114" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G114" s="14">
         <v>0.1</v>
       </c>
       <c r="H114" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I114" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J114" s="15">
         <f t="shared" si="4"/>
@@ -6866,16 +6866,16 @@
         <v>207</v>
       </c>
       <c r="F115" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G115" s="14">
         <v>0.4</v>
       </c>
       <c r="H115" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I115" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J115" s="15">
         <f t="shared" si="4"/>
@@ -6914,16 +6914,16 @@
         <v>207</v>
       </c>
       <c r="F116" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G116" s="14">
         <v>0.48</v>
       </c>
       <c r="H116" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J116" s="15">
         <f t="shared" si="4"/>
@@ -6962,16 +6962,16 @@
         <v>146</v>
       </c>
       <c r="F117" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G117" s="14">
         <v>1112.3900000000001</v>
       </c>
       <c r="H117" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I117" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J117" s="15">
         <f t="shared" si="4"/>
@@ -7010,16 +7010,16 @@
         <v>146</v>
       </c>
       <c r="F118" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G118" s="14">
         <v>1112.3900000000001</v>
       </c>
       <c r="H118" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I118" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J118" s="15">
         <f t="shared" si="4"/>
@@ -7058,16 +7058,16 @@
         <v>207</v>
       </c>
       <c r="F119" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G119" s="14">
         <v>0.24</v>
       </c>
       <c r="H119" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I119" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J119" s="15">
         <f t="shared" si="4"/>
@@ -7106,16 +7106,16 @@
         <v>207</v>
       </c>
       <c r="F120" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G120" s="14">
         <v>10.76</v>
       </c>
       <c r="H120" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I120" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J120" s="15">
         <f t="shared" si="4"/>
@@ -7154,16 +7154,16 @@
         <v>215</v>
       </c>
       <c r="F121" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G121" s="14">
         <v>47.1</v>
       </c>
       <c r="H121" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I121" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J121" s="15">
         <f t="shared" si="4"/>
@@ -7202,16 +7202,16 @@
         <v>207</v>
       </c>
       <c r="F122" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G122" s="14">
         <v>2.46</v>
       </c>
       <c r="H122" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I122" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J122" s="15">
         <f t="shared" si="4"/>
@@ -7250,16 +7250,16 @@
         <v>207</v>
       </c>
       <c r="F123" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G123" s="14">
         <v>2.46</v>
       </c>
       <c r="H123" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I123" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J123" s="15">
         <f t="shared" si="4"/>
@@ -7298,16 +7298,16 @@
         <v>219</v>
       </c>
       <c r="F124" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124" s="14">
         <v>96.93</v>
       </c>
       <c r="H124" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I124" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J124" s="15">
         <f t="shared" si="4"/>
@@ -7346,16 +7346,16 @@
         <v>221</v>
       </c>
       <c r="F125" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G125" s="14">
         <v>96.26</v>
       </c>
       <c r="H125" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I125" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J125" s="15">
         <f t="shared" si="4"/>
@@ -7394,16 +7394,16 @@
         <v>223</v>
       </c>
       <c r="F126" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G126" s="14">
         <v>96.26</v>
       </c>
       <c r="H126" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I126" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J126" s="15">
         <f t="shared" si="4"/>
@@ -7442,16 +7442,16 @@
         <v>195</v>
       </c>
       <c r="F127" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G127" s="14">
         <v>111.93</v>
       </c>
       <c r="H127" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I127" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127" s="15">
         <f t="shared" si="4"/>

</xml_diff>